<commit_message>
all estimates send to nabin sir
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/thekka/Khanal tol khanepaani/khanal tol khanepaani for nabin sir.xlsx
+++ b/बजेट माग estimate/thekka/Khanal tol khanepaani/khanal tol khanepaani for nabin sir.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2CCD2C-5E8B-49BE-8E53-4291B51E0928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802D075C-123B-4E66-9AE2-B0D095C62D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="89">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -117,24 +117,9 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Budget allocated</t>
-  </si>
-  <si>
-    <t>Municipal payment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contingencies </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintanince </t>
-  </si>
-  <si>
     <t>F.Y.: 2082/2083</t>
   </si>
   <si>
-    <t>User contribution</t>
-  </si>
-  <si>
     <t>Length (m)</t>
   </si>
   <si>
@@ -159,9 +144,6 @@
     <t>Location:- Shankharapur Municipality 1</t>
   </si>
   <si>
-    <t>-13% VAT for material</t>
-  </si>
-  <si>
     <t>-for pipe laying</t>
   </si>
   <si>
@@ -180,18 +162,9 @@
     <t>Pipe works</t>
   </si>
   <si>
-    <t>-13% VAT for sand</t>
-  </si>
-  <si>
     <t>Plain cement concrete (1:2:4)</t>
   </si>
   <si>
-    <t>-13% VAT for cement</t>
-  </si>
-  <si>
-    <t>-13% VAT for aggregate</t>
-  </si>
-  <si>
     <t>sqm</t>
   </si>
   <si>
@@ -213,9 +186,6 @@
     <t>3 mm thick  cement punning</t>
   </si>
   <si>
-    <t>-13% VAT for block stone</t>
-  </si>
-  <si>
     <t>thickness</t>
   </si>
   <si>
@@ -226,9 +196,6 @@
   </si>
   <si>
     <t>Total Weight (Kg)</t>
-  </si>
-  <si>
-    <t>-13% VAT for nails</t>
   </si>
   <si>
     <t>Earthwork in Excavation in ordinary soil</t>
@@ -268,16 +235,7 @@
     <t>Kg</t>
   </si>
   <si>
-    <t>-13% VAT for MS bars</t>
-  </si>
-  <si>
-    <t>-13% VAT for Bind wire</t>
-  </si>
-  <si>
     <t>Form work for concrete work</t>
-  </si>
-  <si>
-    <t>-13% VAT for local wood</t>
   </si>
   <si>
     <t>-for 25mm pipe laying from intake to sim intake</t>
@@ -567,7 +525,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -691,6 +649,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -712,21 +676,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1254,7 +1203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA127"/>
+  <dimension ref="A1:AA104"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="4" customWidth="1"/>
@@ -1272,113 +1221,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
     </row>
     <row r="2" spans="1:27" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52"/>
-      <c r="K2" s="52"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
-      <c r="H3" s="53"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="53"/>
-      <c r="K3" s="53"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="55"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53"/>
-      <c r="K4" s="53"/>
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="55"/>
     </row>
     <row r="5" spans="1:27" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="56"/>
     </row>
     <row r="6" spans="1:27" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="55" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="55"/>
-      <c r="C6" s="55"/>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="55"/>
+      <c r="A6" s="57" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="57"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="56" t="s">
-        <v>25</v>
-      </c>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
-      <c r="K6" s="56"/>
+      <c r="H6" s="58" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="58"/>
+      <c r="J6" s="58"/>
+      <c r="K6" s="58"/>
     </row>
     <row r="7" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
+      <c r="A7" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="51"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="51"/>
+      <c r="E7" s="51"/>
+      <c r="F7" s="51"/>
       <c r="G7" s="6"/>
-      <c r="H7" s="50" t="s">
-        <v>55</v>
-      </c>
-      <c r="I7" s="50"/>
-      <c r="J7" s="50"/>
-      <c r="K7" s="50"/>
+      <c r="H7" s="52" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="52"/>
     </row>
     <row r="8" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
@@ -1421,7 +1370,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="14"/>
@@ -1437,7 +1386,7 @@
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="17"/>
       <c r="B10" s="18" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="C10" s="19">
         <v>1</v>
@@ -1464,7 +1413,7 @@
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="18" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="C11" s="19">
         <v>1</v>
@@ -1491,7 +1440,7 @@
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="18" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="C12" s="21">
         <v>0.5</v>
@@ -1518,7 +1467,7 @@
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
       <c r="B13" s="18" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="C13" s="21">
         <v>1</v>
@@ -1556,14 +1505,15 @@
         <v>11.862925727674487</v>
       </c>
       <c r="H14" s="26" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="I14" s="2">
-        <v>963.05</v>
+        <f>1.15*963.05</f>
+        <v>1107.5074999999999</v>
       </c>
       <c r="J14" s="27">
         <f>G14*I14</f>
-        <v>11424.590622036914</v>
+        <v>13138.279215342451</v>
       </c>
       <c r="K14" s="25"/>
     </row>
@@ -1585,7 +1535,7 @@
         <v>2</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -1724,23 +1674,21 @@
         <v>2.5146819776744893</v>
       </c>
       <c r="H21" s="26" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="I21" s="2">
-        <f>4493.69</f>
-        <v>4493.6899999999996</v>
+        <f>1.15*4493.69</f>
+        <v>5167.7434999999996</v>
       </c>
       <c r="J21" s="27">
         <f>G21*I21</f>
-        <v>11300.201256256074</v>
+        <v>12995.231444694486</v>
       </c>
       <c r="K21" s="25"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="17"/>
-      <c r="B22" s="18" t="s">
-        <v>53</v>
-      </c>
+      <c r="B22" s="19"/>
       <c r="C22" s="19"/>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
@@ -1748,15 +1696,16 @@
       <c r="G22" s="19"/>
       <c r="H22" s="19"/>
       <c r="I22" s="19"/>
-      <c r="J22" s="27">
-        <f>0.13*G21*3091.19</f>
-        <v>1010.5367717337887</v>
-      </c>
+      <c r="J22" s="19"/>
       <c r="K22" s="19"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="17"/>
-      <c r="B23" s="19"/>
+      <c r="A23" s="17">
+        <v>3</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>36</v>
+      </c>
       <c r="C23" s="19"/>
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
@@ -1768,17 +1717,28 @@
       <c r="K23" s="19"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="17">
-        <v>3</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
+      <c r="A24" s="17"/>
+      <c r="B24" s="18" t="str">
+        <f>B10</f>
+        <v>-for intake 1</v>
+      </c>
+      <c r="C24" s="19">
+        <f>C10</f>
+        <v>1</v>
+      </c>
+      <c r="D24" s="20">
+        <v>1.8</v>
+      </c>
+      <c r="E24" s="20">
+        <v>1.8</v>
+      </c>
+      <c r="F24" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="G24" s="20">
+        <f>PRODUCT(C24:F24)</f>
+        <v>0.32400000000000007</v>
+      </c>
       <c r="H24" s="19"/>
       <c r="I24" s="19"/>
       <c r="J24" s="19"/>
@@ -1787,25 +1747,25 @@
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="17"/>
       <c r="B25" s="18" t="str">
-        <f>B10</f>
-        <v>-for intake 1</v>
+        <f>B11</f>
+        <v>-for intake 2</v>
       </c>
       <c r="C25" s="19">
-        <f>C10</f>
+        <f>C11</f>
         <v>1</v>
       </c>
       <c r="D25" s="20">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E25" s="20">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="F25" s="20">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G25" s="20">
         <f>PRODUCT(C25:F25)</f>
-        <v>0.32400000000000007</v>
+        <v>0.2</v>
       </c>
       <c r="H25" s="19"/>
       <c r="I25" s="19"/>
@@ -1815,25 +1775,25 @@
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="17"/>
       <c r="B26" s="18" t="str">
-        <f>B11</f>
-        <v>-for intake 2</v>
-      </c>
-      <c r="C26" s="19">
-        <f>C11</f>
-        <v>1</v>
+        <f>B19</f>
+        <v>-for kulo</v>
+      </c>
+      <c r="C26" s="21">
+        <f>C19</f>
+        <v>0.5</v>
       </c>
       <c r="D26" s="20">
-        <v>2</v>
+        <v>21.335000000000001</v>
       </c>
       <c r="E26" s="20">
-        <v>2</v>
-      </c>
-      <c r="F26" s="20">
-        <v>0.05</v>
+        <v>0.54999999999999993</v>
+      </c>
+      <c r="F26" s="19">
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="G26" s="20">
         <f>PRODUCT(C26:F26)</f>
-        <v>0.2</v>
+        <v>0.44003437499999998</v>
       </c>
       <c r="H26" s="19"/>
       <c r="I26" s="19"/>
@@ -1843,90 +1803,78 @@
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="17"/>
       <c r="B27" s="18" t="str">
-        <f>B19</f>
-        <v>-for kulo</v>
+        <f>B20</f>
+        <v>-for kulo 2</v>
       </c>
       <c r="C27" s="21">
-        <f>C19</f>
-        <v>0.5</v>
+        <f>C20</f>
+        <v>1</v>
       </c>
       <c r="D27" s="20">
-        <v>21.335000000000001</v>
+        <f>D20</f>
+        <v>12.1914050594331</v>
       </c>
       <c r="E27" s="20">
-        <v>0.54999999999999993</v>
+        <f>E20</f>
+        <v>0.3</v>
       </c>
       <c r="F27" s="19">
-        <v>7.4999999999999997E-2</v>
+        <v>0.1</v>
       </c>
       <c r="G27" s="20">
         <f>PRODUCT(C27:F27)</f>
-        <v>0.44003437499999998</v>
+        <v>0.36574215178299302</v>
       </c>
       <c r="H27" s="19"/>
       <c r="I27" s="19"/>
       <c r="J27" s="19"/>
       <c r="K27" s="19"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="17"/>
-      <c r="B28" s="18" t="str">
-        <f>B20</f>
-        <v>-for kulo 2</v>
-      </c>
-      <c r="C28" s="21">
-        <f>C20</f>
-        <v>1</v>
-      </c>
-      <c r="D28" s="20">
-        <f>D20</f>
-        <v>12.1914050594331</v>
-      </c>
-      <c r="E28" s="20">
-        <f>E20</f>
-        <v>0.3</v>
-      </c>
-      <c r="F28" s="19">
-        <v>0.1</v>
-      </c>
-      <c r="G28" s="20">
-        <f>PRODUCT(C28:F28)</f>
-        <v>0.36574215178299302</v>
-      </c>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-    </row>
-    <row r="29" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="22"/>
-      <c r="B29" s="23" t="s">
+    <row r="28" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="22"/>
+      <c r="B28" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="24"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="2">
-        <f>SUM(G25:G28)</f>
+      <c r="C28" s="24"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="2">
+        <f>SUM(G24:G27)</f>
         <v>1.3297765267829931</v>
       </c>
-      <c r="H29" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="I29" s="2">
-        <v>13343.7</v>
-      </c>
-      <c r="J29" s="27">
-        <f>G29*I29</f>
-        <v>17744.139040434227</v>
-      </c>
-      <c r="K29" s="25"/>
+      <c r="H28" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="I28" s="2">
+        <f>1.15*13343.7</f>
+        <v>15345.254999999999</v>
+      </c>
+      <c r="J28" s="27">
+        <f>G28*I28</f>
+        <v>20405.759896499356</v>
+      </c>
+      <c r="K28" s="25"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="17"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="19"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="17"/>
-      <c r="B30" s="18" t="s">
-        <v>42</v>
+      <c r="A30" s="17">
+        <v>4</v>
+      </c>
+      <c r="B30" s="28" t="s">
+        <v>62</v>
       </c>
       <c r="C30" s="19"/>
       <c r="D30" s="19"/>
@@ -1935,68 +1883,90 @@
       <c r="G30" s="19"/>
       <c r="H30" s="19"/>
       <c r="I30" s="19"/>
-      <c r="J30" s="27">
-        <f>0.13*G29*1413.27</f>
-        <v>244.31332536085807</v>
-      </c>
+      <c r="J30" s="19"/>
       <c r="K30" s="19"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="17"/>
       <c r="B31" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
+        <v>64</v>
+      </c>
+      <c r="C31" s="19">
+        <f>C24*2</f>
+        <v>2</v>
+      </c>
+      <c r="D31" s="20">
+        <v>1.8</v>
+      </c>
+      <c r="E31" s="20">
+        <v>0.45</v>
+      </c>
+      <c r="F31" s="20">
+        <v>0.9</v>
+      </c>
+      <c r="G31" s="20">
+        <v>1.4580000000000002</v>
+      </c>
       <c r="H31" s="19"/>
       <c r="I31" s="19"/>
-      <c r="J31" s="27">
-        <f>0.13*G29*4096</f>
-        <v>708.07940498140817</v>
-      </c>
+      <c r="J31" s="19"/>
       <c r="K31" s="19"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="17"/>
       <c r="B32" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
+        <v>65</v>
+      </c>
+      <c r="C32" s="19">
+        <f>C24*2</f>
+        <v>2</v>
+      </c>
+      <c r="D32" s="20">
+        <v>0.90000000000000013</v>
+      </c>
+      <c r="E32" s="20">
+        <v>0.45</v>
+      </c>
+      <c r="F32" s="20">
+        <v>0.9</v>
+      </c>
+      <c r="G32" s="20">
+        <v>0.7290000000000002</v>
+      </c>
       <c r="H32" s="19"/>
       <c r="I32" s="19"/>
-      <c r="J32" s="27">
-        <f>0.13*G29*(368.76+737.51+1743.21)</f>
-        <v>492.59231027988841</v>
-      </c>
+      <c r="J32" s="19"/>
       <c r="K32" s="19"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="17"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
-    </row>
-    <row r="34" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="17">
-        <v>4</v>
-      </c>
-      <c r="B34" s="28" t="s">
-        <v>76</v>
-      </c>
+    <row r="33" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="22"/>
+      <c r="B33" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="24"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="2">
+        <f>SUM(G31:G32)</f>
+        <v>2.1870000000000003</v>
+      </c>
+      <c r="H33" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="I33" s="2">
+        <f>1.15*12225.55</f>
+        <v>14059.382499999998</v>
+      </c>
+      <c r="J33" s="27">
+        <f>G33*I33</f>
+        <v>30747.869527499999</v>
+      </c>
+      <c r="K33" s="25"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="17"/>
+      <c r="B34" s="19"/>
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
       <c r="E34" s="19"/>
@@ -2008,26 +1978,17 @@
       <c r="K34" s="19"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="17"/>
-      <c r="B35" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="C35" s="19">
-        <f>C25*2</f>
-        <v>2</v>
-      </c>
-      <c r="D35" s="20">
-        <v>1.8</v>
-      </c>
-      <c r="E35" s="20">
-        <v>0.45</v>
-      </c>
-      <c r="F35" s="20">
-        <v>0.9</v>
-      </c>
-      <c r="G35" s="20">
-        <v>1.4580000000000002</v>
-      </c>
+      <c r="A35" s="17">
+        <v>5</v>
+      </c>
+      <c r="B35" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
       <c r="H35" s="19"/>
       <c r="I35" s="19"/>
       <c r="J35" s="19"/>
@@ -2036,107 +1997,128 @@
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="17"/>
       <c r="B36" s="18" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="C36" s="19">
-        <f>C25*2</f>
-        <v>2</v>
+        <f>C24</f>
+        <v>1</v>
       </c>
       <c r="D36" s="20">
-        <v>0.90000000000000013</v>
-      </c>
-      <c r="E36" s="20">
-        <v>0.45</v>
-      </c>
+        <v>7.2</v>
+      </c>
+      <c r="E36" s="20"/>
       <c r="F36" s="20">
         <v>0.9</v>
       </c>
       <c r="G36" s="20">
-        <v>0.7290000000000002</v>
+        <f>PRODUCT(C36:F36)</f>
+        <v>6.48</v>
       </c>
       <c r="H36" s="19"/>
       <c r="I36" s="19"/>
       <c r="J36" s="19"/>
       <c r="K36" s="19"/>
     </row>
-    <row r="37" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="22"/>
-      <c r="B37" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C37" s="24"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="2">
-        <f>SUM(G35:G36)</f>
-        <v>2.1870000000000003</v>
-      </c>
-      <c r="H37" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="I37" s="2">
-        <v>12225.55</v>
-      </c>
-      <c r="J37" s="27">
-        <f>G37*I37</f>
-        <v>26737.277850000002</v>
-      </c>
-      <c r="K37" s="25"/>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="17"/>
+      <c r="B37" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="19">
+        <f>C24</f>
+        <v>1</v>
+      </c>
+      <c r="D37" s="20">
+        <v>3.6000000000000005</v>
+      </c>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20">
+        <v>0.9</v>
+      </c>
+      <c r="G37" s="20">
+        <f>PRODUCT(C37:F37)</f>
+        <v>3.2400000000000007</v>
+      </c>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
+      <c r="J37" s="19"/>
+      <c r="K37" s="19"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="17"/>
       <c r="B38" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
+        <v>84</v>
+      </c>
+      <c r="C38" s="19">
+        <f>C25</f>
+        <v>1</v>
+      </c>
+      <c r="D38" s="20">
+        <v>8</v>
+      </c>
+      <c r="E38" s="20"/>
+      <c r="F38" s="20">
+        <v>1.2</v>
+      </c>
+      <c r="G38" s="20">
+        <f>PRODUCT(C38:F38)</f>
+        <v>9.6</v>
+      </c>
       <c r="H38" s="19"/>
       <c r="I38" s="19"/>
-      <c r="J38" s="27">
-        <f>0.13*G37*1492.66</f>
-        <v>424.3781646000001</v>
-      </c>
+      <c r="J38" s="19"/>
       <c r="K38" s="19"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="17"/>
       <c r="B39" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
+        <v>85</v>
+      </c>
+      <c r="C39" s="19">
+        <f>C25</f>
+        <v>1</v>
+      </c>
+      <c r="D39" s="20">
+        <v>7.1999999999999993</v>
+      </c>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20">
+        <v>1.2</v>
+      </c>
+      <c r="G39" s="20">
+        <f>PRODUCT(C39:F39)</f>
+        <v>8.6399999999999988</v>
+      </c>
       <c r="H39" s="19"/>
       <c r="I39" s="19"/>
-      <c r="J39" s="27">
-        <f>0.13*G37*1356.8</f>
-        <v>385.7518080000001</v>
-      </c>
+      <c r="J39" s="19"/>
       <c r="K39" s="19"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="17"/>
-      <c r="B40" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="C40" s="19"/>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="19"/>
+    <row r="40" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="22"/>
+      <c r="B40" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="24"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="2">
+        <f>SUM(G36:G39)</f>
+        <v>27.96</v>
+      </c>
+      <c r="H40" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="I40" s="2">
+        <f>1.15*49954.32/100</f>
+        <v>574.47467999999992</v>
+      </c>
       <c r="J40" s="27">
-        <f>0.13*G37*2833.59</f>
-        <v>805.61797290000027</v>
-      </c>
-      <c r="K40" s="19"/>
+        <f>G40*I40</f>
+        <v>16062.312052799998</v>
+      </c>
+      <c r="K40" s="25"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="17"/>
@@ -2153,10 +2135,10 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B42" s="28" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="19"/>
@@ -2170,15 +2152,16 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="17"/>
-      <c r="B43" s="18" t="s">
-        <v>80</v>
+      <c r="B43" s="18" t="str">
+        <f>B37</f>
+        <v>-for inner face wall of intake 1</v>
       </c>
       <c r="C43" s="19">
-        <f>C25</f>
+        <f>C37</f>
         <v>1</v>
       </c>
       <c r="D43" s="20">
-        <v>7.2</v>
+        <v>3.6000000000000005</v>
       </c>
       <c r="E43" s="20"/>
       <c r="F43" s="20">
@@ -2186,7 +2169,7 @@
       </c>
       <c r="G43" s="20">
         <f>PRODUCT(C43:F43)</f>
-        <v>6.48</v>
+        <v>3.2400000000000007</v>
       </c>
       <c r="H43" s="19"/>
       <c r="I43" s="19"/>
@@ -2196,22 +2179,22 @@
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="17"/>
       <c r="B44" s="18" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="C44" s="19">
-        <f>C25</f>
+        <f>C43</f>
         <v>1</v>
       </c>
       <c r="D44" s="20">
-        <v>3.6000000000000005</v>
-      </c>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20">
-        <v>0.9</v>
-      </c>
+        <v>0.90000000000000013</v>
+      </c>
+      <c r="E44" s="20">
+        <v>0.90000000000000013</v>
+      </c>
+      <c r="F44" s="20"/>
       <c r="G44" s="20">
         <f>PRODUCT(C44:F44)</f>
-        <v>3.2400000000000007</v>
+        <v>0.81000000000000028</v>
       </c>
       <c r="H44" s="19"/>
       <c r="I44" s="19"/>
@@ -2220,15 +2203,16 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="17"/>
-      <c r="B45" s="18" t="s">
-        <v>98</v>
+      <c r="B45" s="18" t="str">
+        <f>B39</f>
+        <v>-for inner face wall of intake 2</v>
       </c>
       <c r="C45" s="19">
-        <f>C26</f>
+        <f>C39</f>
         <v>1</v>
       </c>
       <c r="D45" s="20">
-        <v>8</v>
+        <v>7.1999999999999993</v>
       </c>
       <c r="E45" s="20"/>
       <c r="F45" s="20">
@@ -2236,7 +2220,7 @@
       </c>
       <c r="G45" s="20">
         <f>PRODUCT(C45:F45)</f>
-        <v>9.6</v>
+        <v>8.6399999999999988</v>
       </c>
       <c r="H45" s="19"/>
       <c r="I45" s="19"/>
@@ -2246,22 +2230,22 @@
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="17"/>
       <c r="B46" s="18" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="C46" s="19">
-        <f>C26</f>
+        <f>C45</f>
         <v>1</v>
       </c>
       <c r="D46" s="20">
-        <v>7.1999999999999993</v>
-      </c>
-      <c r="E46" s="20"/>
-      <c r="F46" s="20">
-        <v>1.2</v>
-      </c>
+        <v>1.7999999999999998</v>
+      </c>
+      <c r="E46" s="20">
+        <v>1.7999999999999998</v>
+      </c>
+      <c r="F46" s="20"/>
       <c r="G46" s="20">
         <f>PRODUCT(C46:F46)</f>
-        <v>8.6399999999999988</v>
+        <v>3.2399999999999993</v>
       </c>
       <c r="H46" s="19"/>
       <c r="I46" s="19"/>
@@ -2279,26 +2263,24 @@
       <c r="F47" s="25"/>
       <c r="G47" s="2">
         <f>SUM(G43:G46)</f>
-        <v>27.96</v>
+        <v>15.93</v>
       </c>
       <c r="H47" s="26" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="I47" s="2">
-        <f>49954.32/100</f>
-        <v>499.54320000000001</v>
+        <f>1.15*28609.6/100</f>
+        <v>329.01039999999995</v>
       </c>
       <c r="J47" s="27">
         <f>G47*I47</f>
-        <v>13967.227872000001</v>
+        <v>5241.1356719999994</v>
       </c>
       <c r="K47" s="25"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="17"/>
-      <c r="B48" s="18" t="s">
-        <v>42</v>
-      </c>
+      <c r="B48" s="19"/>
       <c r="C48" s="19"/>
       <c r="D48" s="19"/>
       <c r="E48" s="19"/>
@@ -2306,33 +2288,42 @@
       <c r="G48" s="19"/>
       <c r="H48" s="19"/>
       <c r="I48" s="19"/>
-      <c r="J48" s="27">
-        <f>0.13*G47*7463.32/100</f>
-        <v>271.27675536000004</v>
-      </c>
+      <c r="J48" s="19"/>
       <c r="K48" s="19"/>
     </row>
-    <row r="49" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A49" s="17"/>
-      <c r="B49" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="19"/>
-      <c r="G49" s="19"/>
-      <c r="H49" s="19"/>
-      <c r="I49" s="19"/>
-      <c r="J49" s="27">
-        <f>0.13*G47*7296/100</f>
-        <v>265.19500800000003</v>
-      </c>
-      <c r="K49" s="19"/>
+    <row r="49" spans="1:27" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A49" s="22">
+        <v>7</v>
+      </c>
+      <c r="B49" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="C49" s="24">
+        <v>1</v>
+      </c>
+      <c r="D49" s="1"/>
+      <c r="E49" s="25"/>
+      <c r="F49" s="25"/>
+      <c r="G49" s="30">
+        <f>PRODUCT(C49:F49)</f>
+        <v>1</v>
+      </c>
+      <c r="H49" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="I49" s="2">
+        <v>3000</v>
+      </c>
+      <c r="J49" s="30">
+        <f>G49*I49</f>
+        <v>3000</v>
+      </c>
+      <c r="K49" s="25"/>
+      <c r="AA49" s="4"/>
     </row>
     <row r="50" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A50" s="17"/>
-      <c r="B50" s="19"/>
+      <c r="B50" s="13"/>
       <c r="C50" s="19"/>
       <c r="D50" s="19"/>
       <c r="E50" s="19"/>
@@ -2345,10 +2336,10 @@
     </row>
     <row r="51" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A51" s="17">
-        <v>6</v>
-      </c>
-      <c r="B51" s="28" t="s">
-        <v>52</v>
+        <v>8</v>
+      </c>
+      <c r="B51" s="19" t="s">
+        <v>55</v>
       </c>
       <c r="C51" s="19"/>
       <c r="D51" s="19"/>
@@ -2362,24 +2353,22 @@
     </row>
     <row r="52" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A52" s="17"/>
-      <c r="B52" s="18" t="str">
-        <f>B44</f>
-        <v>-for inner face wall of intake 1</v>
+      <c r="B52" s="18" t="s">
+        <v>69</v>
       </c>
       <c r="C52" s="19">
-        <f>C44</f>
         <v>1</v>
       </c>
       <c r="D52" s="20">
-        <v>3.6000000000000005</v>
+        <v>7.2</v>
       </c>
       <c r="E52" s="20"/>
       <c r="F52" s="20">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="G52" s="20">
-        <f>PRODUCT(C52:F52)</f>
-        <v>3.2400000000000007</v>
+        <f t="shared" ref="G52:G57" si="0">PRODUCT(C52:F52)</f>
+        <v>0.72000000000000008</v>
       </c>
       <c r="H52" s="19"/>
       <c r="I52" s="19"/>
@@ -2389,22 +2378,21 @@
     <row r="53" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A53" s="17"/>
       <c r="B53" s="18" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C53" s="19">
-        <f>C52</f>
         <v>1</v>
       </c>
       <c r="D53" s="20">
-        <v>0.90000000000000013</v>
-      </c>
-      <c r="E53" s="20">
-        <v>0.90000000000000013</v>
-      </c>
-      <c r="F53" s="20"/>
+        <v>8</v>
+      </c>
+      <c r="E53" s="20"/>
+      <c r="F53" s="20">
+        <v>1.2</v>
+      </c>
       <c r="G53" s="20">
-        <f>PRODUCT(C53:F53)</f>
-        <v>0.81000000000000028</v>
+        <f t="shared" si="0"/>
+        <v>9.6</v>
       </c>
       <c r="H53" s="19"/>
       <c r="I53" s="19"/>
@@ -2413,12 +2401,10 @@
     </row>
     <row r="54" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A54" s="17"/>
-      <c r="B54" s="18" t="str">
-        <f>B46</f>
-        <v>-for inner face wall of intake 2</v>
+      <c r="B54" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="C54" s="19">
-        <f>C46</f>
         <v>1</v>
       </c>
       <c r="D54" s="20">
@@ -2429,7 +2415,7 @@
         <v>1.2</v>
       </c>
       <c r="G54" s="20">
-        <f>PRODUCT(C54:F54)</f>
+        <f t="shared" si="0"/>
         <v>8.6399999999999988</v>
       </c>
       <c r="H54" s="19"/>
@@ -2440,10 +2426,9 @@
     <row r="55" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A55" s="17"/>
       <c r="B55" s="18" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="C55" s="19">
-        <f>C54</f>
         <v>1</v>
       </c>
       <c r="D55" s="20">
@@ -2454,7 +2439,7 @@
       </c>
       <c r="F55" s="20"/>
       <c r="G55" s="20">
-        <f>PRODUCT(C55:F55)</f>
+        <f t="shared" si="0"/>
         <v>3.2399999999999993</v>
       </c>
       <c r="H55" s="19"/>
@@ -2462,96 +2447,106 @@
       <c r="J55" s="19"/>
       <c r="K55" s="19"/>
     </row>
-    <row r="56" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="22"/>
-      <c r="B56" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C56" s="24"/>
-      <c r="D56" s="1"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="25"/>
-      <c r="G56" s="2">
-        <f>SUM(G52:G55)</f>
-        <v>15.93</v>
-      </c>
-      <c r="H56" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="I56" s="2">
-        <f>28609.6/100</f>
-        <v>286.096</v>
-      </c>
-      <c r="J56" s="27">
-        <f>G56*I56</f>
-        <v>4557.5092800000002</v>
-      </c>
-      <c r="K56" s="25"/>
+    <row r="56" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A56" s="17"/>
+      <c r="B56" s="18" t="str">
+        <f>B67</f>
+        <v>-for kulo shear wall</v>
+      </c>
+      <c r="C56" s="19">
+        <f>C67*2</f>
+        <v>4</v>
+      </c>
+      <c r="D56" s="20">
+        <f>D67</f>
+        <v>21.34</v>
+      </c>
+      <c r="E56" s="20"/>
+      <c r="F56" s="20">
+        <f>F67</f>
+        <v>0.45</v>
+      </c>
+      <c r="G56" s="20">
+        <f t="shared" si="0"/>
+        <v>38.411999999999999</v>
+      </c>
+      <c r="H56" s="19"/>
+      <c r="I56" s="19"/>
+      <c r="J56" s="19"/>
+      <c r="K56" s="19"/>
     </row>
     <row r="57" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A57" s="17"/>
-      <c r="B57" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C57" s="19"/>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="19"/>
-      <c r="G57" s="19"/>
+      <c r="B57" s="18" t="str">
+        <f>B68</f>
+        <v>-for shear wall cover slab</v>
+      </c>
+      <c r="C57" s="19">
+        <f>TRUNC(D56/0.6,0)</f>
+        <v>35</v>
+      </c>
+      <c r="D57" s="20">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E57" s="20"/>
+      <c r="F57" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="G57" s="20">
+        <f t="shared" si="0"/>
+        <v>8.0500000000000007</v>
+      </c>
       <c r="H57" s="19"/>
       <c r="I57" s="19"/>
-      <c r="J57" s="27">
-        <f>0.13*G56*6809.6/100</f>
-        <v>141.0200064</v>
-      </c>
+      <c r="J57" s="19"/>
       <c r="K57" s="19"/>
     </row>
-    <row r="58" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A58" s="17"/>
-      <c r="B58" s="19"/>
-      <c r="C58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="19"/>
-      <c r="I58" s="19"/>
-      <c r="J58" s="19"/>
-      <c r="K58" s="19"/>
-    </row>
-    <row r="59" spans="1:27" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A59" s="22">
-        <v>7</v>
-      </c>
-      <c r="B59" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="C59" s="24">
-        <v>1</v>
-      </c>
-      <c r="D59" s="1"/>
-      <c r="E59" s="25"/>
-      <c r="F59" s="25"/>
-      <c r="G59" s="30">
-        <f>PRODUCT(C59:F59)</f>
-        <v>1</v>
-      </c>
-      <c r="H59" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="I59" s="2">
-        <v>3000</v>
-      </c>
-      <c r="J59" s="30">
-        <f>G59*I59</f>
-        <v>3000</v>
-      </c>
-      <c r="K59" s="25"/>
-      <c r="AA59" s="4"/>
+    <row r="58" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="22"/>
+      <c r="B58" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C58" s="24"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="25"/>
+      <c r="F58" s="25"/>
+      <c r="G58" s="2">
+        <f>SUM(G52:G57)</f>
+        <v>68.661999999999992</v>
+      </c>
+      <c r="H58" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="I58" s="2">
+        <f>1.15*11188.35/10</f>
+        <v>1286.6602499999999</v>
+      </c>
+      <c r="J58" s="27">
+        <f>G58*I58</f>
+        <v>88344.666085499979</v>
+      </c>
+      <c r="K58" s="25"/>
+    </row>
+    <row r="59" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A59" s="17"/>
+      <c r="B59" s="19"/>
+      <c r="C59" s="19"/>
+      <c r="D59" s="19"/>
+      <c r="E59" s="19"/>
+      <c r="F59" s="19"/>
+      <c r="G59" s="19"/>
+      <c r="H59" s="19"/>
+      <c r="I59" s="19"/>
+      <c r="J59" s="19"/>
+      <c r="K59" s="19"/>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A60" s="17"/>
-      <c r="B60" s="13"/>
+      <c r="A60" s="17">
+        <v>9</v>
+      </c>
+      <c r="B60" s="19" t="s">
+        <v>52</v>
+      </c>
       <c r="C60" s="19"/>
       <c r="D60" s="19"/>
       <c r="E60" s="19"/>
@@ -2563,17 +2558,27 @@
       <c r="K60" s="19"/>
     </row>
     <row r="61" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A61" s="17">
-        <v>8</v>
-      </c>
-      <c r="B61" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="C61" s="19"/>
-      <c r="D61" s="19"/>
-      <c r="E61" s="19"/>
-      <c r="F61" s="19"/>
-      <c r="G61" s="19"/>
+      <c r="A61" s="17"/>
+      <c r="B61" s="18" t="str">
+        <f>B52</f>
+        <v>-for intake 1 cover</v>
+      </c>
+      <c r="C61" s="19">
+        <v>1</v>
+      </c>
+      <c r="D61" s="20">
+        <v>1.8</v>
+      </c>
+      <c r="E61" s="20">
+        <v>1.8</v>
+      </c>
+      <c r="F61" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="G61" s="20">
+        <f t="shared" ref="G61:G68" si="1">PRODUCT(C61:F61)</f>
+        <v>0.32400000000000007</v>
+      </c>
       <c r="H61" s="19"/>
       <c r="I61" s="19"/>
       <c r="J61" s="19"/>
@@ -2581,22 +2586,25 @@
     </row>
     <row r="62" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A62" s="17"/>
-      <c r="B62" s="18" t="s">
-        <v>83</v>
+      <c r="B62" s="18" t="str">
+        <f>B18</f>
+        <v>-for intake 2</v>
       </c>
       <c r="C62" s="19">
         <v>1</v>
       </c>
       <c r="D62" s="20">
-        <v>7.2</v>
-      </c>
-      <c r="E62" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="E62" s="20">
+        <v>2</v>
+      </c>
       <c r="F62" s="20">
         <v>0.1</v>
       </c>
       <c r="G62" s="20">
-        <f t="shared" ref="G62:G67" si="0">PRODUCT(C62:F62)</f>
-        <v>0.72000000000000008</v>
+        <f t="shared" si="1"/>
+        <v>0.4</v>
       </c>
       <c r="H62" s="19"/>
       <c r="I62" s="19"/>
@@ -2606,21 +2614,23 @@
     <row r="63" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A63" s="17"/>
       <c r="B63" s="18" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="C63" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D63" s="20">
-        <v>8</v>
-      </c>
-      <c r="E63" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="E63" s="20">
+        <v>0.1</v>
+      </c>
       <c r="F63" s="20">
         <v>1.2</v>
       </c>
       <c r="G63" s="20">
-        <f t="shared" si="0"/>
-        <v>9.6</v>
+        <f t="shared" si="1"/>
+        <v>0.48</v>
       </c>
       <c r="H63" s="19"/>
       <c r="I63" s="19"/>
@@ -2630,21 +2640,23 @@
     <row r="64" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A64" s="17"/>
       <c r="B64" s="18" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="C64" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64" s="20">
-        <v>7.1999999999999993</v>
-      </c>
-      <c r="E64" s="20"/>
+        <v>1.7999999999999998</v>
+      </c>
+      <c r="E64" s="20">
+        <v>0.1</v>
+      </c>
       <c r="F64" s="20">
         <v>1.2</v>
       </c>
       <c r="G64" s="20">
-        <f t="shared" si="0"/>
-        <v>8.6399999999999988</v>
+        <f t="shared" si="1"/>
+        <v>0.432</v>
       </c>
       <c r="H64" s="19"/>
       <c r="I64" s="19"/>
@@ -2653,22 +2665,25 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="17"/>
-      <c r="B65" s="18" t="s">
-        <v>91</v>
+      <c r="B65" s="18" t="str">
+        <f>B55</f>
+        <v>-for intake 2 cover</v>
       </c>
       <c r="C65" s="19">
         <v>1</v>
       </c>
       <c r="D65" s="20">
-        <v>1.7999999999999998</v>
+        <v>2</v>
       </c>
       <c r="E65" s="20">
-        <v>1.7999999999999998</v>
-      </c>
-      <c r="F65" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="F65" s="20">
+        <v>0.1</v>
+      </c>
       <c r="G65" s="20">
-        <f t="shared" si="0"/>
-        <v>3.2399999999999993</v>
+        <f t="shared" si="1"/>
+        <v>0.4</v>
       </c>
       <c r="H65" s="19"/>
       <c r="I65" s="19"/>
@@ -2677,26 +2692,27 @@
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="17"/>
-      <c r="B66" s="18" t="str">
-        <f>B79</f>
-        <v>-for kulo shear wall</v>
-      </c>
-      <c r="C66" s="19">
-        <f>C79*2</f>
-        <v>4</v>
+      <c r="B66" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C66" s="21">
+        <f>C26</f>
+        <v>0.5</v>
       </c>
       <c r="D66" s="20">
-        <f>D79</f>
-        <v>21.34</v>
-      </c>
-      <c r="E66" s="20"/>
+        <f>D26</f>
+        <v>21.335000000000001</v>
+      </c>
+      <c r="E66" s="20">
+        <f>E26</f>
+        <v>0.54999999999999993</v>
+      </c>
       <c r="F66" s="20">
-        <f>F79</f>
-        <v>0.45</v>
+        <v>0.1</v>
       </c>
       <c r="G66" s="20">
-        <f t="shared" si="0"/>
-        <v>38.411999999999999</v>
+        <f t="shared" si="1"/>
+        <v>0.58671249999999997</v>
       </c>
       <c r="H66" s="19"/>
       <c r="I66" s="19"/>
@@ -2705,79 +2721,85 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="17"/>
-      <c r="B67" s="18" t="str">
-        <f>B80</f>
-        <v>-for shear wall cover slab</v>
-      </c>
-      <c r="C67" s="19">
-        <f>TRUNC(D66/0.6,0)</f>
-        <v>35</v>
+      <c r="B67" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C67" s="21">
+        <v>2</v>
       </c>
       <c r="D67" s="20">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="E67" s="20"/>
+        <v>21.34</v>
+      </c>
+      <c r="E67" s="20">
+        <v>0.1</v>
+      </c>
       <c r="F67" s="20">
-        <v>0.1</v>
+        <v>0.45</v>
       </c>
       <c r="G67" s="20">
-        <f t="shared" si="0"/>
-        <v>8.0500000000000007</v>
+        <f t="shared" si="1"/>
+        <v>1.9205999999999999</v>
       </c>
       <c r="H67" s="19"/>
       <c r="I67" s="19"/>
       <c r="J67" s="19"/>
       <c r="K67" s="19"/>
     </row>
-    <row r="68" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="22"/>
-      <c r="B68" s="23" t="s">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A68" s="17"/>
+      <c r="B68" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C68" s="21">
+        <v>1</v>
+      </c>
+      <c r="D68" s="20">
+        <v>21.34</v>
+      </c>
+      <c r="E68" s="20">
+        <v>0.54999999999999993</v>
+      </c>
+      <c r="F68" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="G68" s="20">
+        <f t="shared" si="1"/>
+        <v>1.1737</v>
+      </c>
+      <c r="H68" s="19"/>
+      <c r="I68" s="19"/>
+      <c r="J68" s="19"/>
+      <c r="K68" s="19"/>
+    </row>
+    <row r="69" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="22"/>
+      <c r="B69" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C68" s="24"/>
-      <c r="D68" s="1"/>
-      <c r="E68" s="25"/>
-      <c r="F68" s="25"/>
-      <c r="G68" s="2">
-        <f>SUM(G62:G67)</f>
-        <v>68.661999999999992</v>
-      </c>
-      <c r="H68" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="I68" s="2">
-        <f>11188.35/10</f>
-        <v>1118.835</v>
-      </c>
-      <c r="J68" s="27">
-        <f>G68*I68</f>
-        <v>76821.448769999988</v>
-      </c>
-      <c r="K68" s="25"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A69" s="17"/>
-      <c r="B69" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C69" s="19"/>
-      <c r="D69" s="19"/>
-      <c r="E69" s="19"/>
-      <c r="F69" s="19"/>
-      <c r="G69" s="19"/>
-      <c r="H69" s="19"/>
-      <c r="I69" s="19"/>
+      <c r="C69" s="24"/>
+      <c r="D69" s="1"/>
+      <c r="E69" s="25"/>
+      <c r="F69" s="25"/>
+      <c r="G69" s="2">
+        <f>SUM(G61:G68)</f>
+        <v>5.7170125000000001</v>
+      </c>
+      <c r="H69" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="I69" s="2">
+        <f>1.15*14337.7</f>
+        <v>16488.355</v>
+      </c>
       <c r="J69" s="27">
-        <f>0.13*G68*6314/10</f>
-        <v>5635.9142840000004</v>
-      </c>
-      <c r="K69" s="19"/>
+        <f>G69*I69</f>
+        <v>94264.131639437503</v>
+      </c>
+      <c r="K69" s="25"/>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="17"/>
-      <c r="B70" s="18" t="s">
-        <v>58</v>
-      </c>
+      <c r="B70" s="19"/>
       <c r="C70" s="19"/>
       <c r="D70" s="19"/>
       <c r="E70" s="19"/>
@@ -2785,37 +2807,60 @@
       <c r="G70" s="19"/>
       <c r="H70" s="19"/>
       <c r="I70" s="19"/>
-      <c r="J70" s="27">
-        <f>0.13*G68*330/10</f>
-        <v>294.55998</v>
-      </c>
+      <c r="J70" s="19"/>
       <c r="K70" s="19"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A71" s="17"/>
-      <c r="B71" s="19"/>
-      <c r="C71" s="19"/>
-      <c r="D71" s="19"/>
-      <c r="E71" s="19"/>
-      <c r="F71" s="19"/>
-      <c r="G71" s="19"/>
-      <c r="H71" s="19"/>
-      <c r="I71" s="19"/>
-      <c r="J71" s="19"/>
-      <c r="K71" s="19"/>
+    <row r="71" spans="1:11" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A71" s="17">
+        <v>10</v>
+      </c>
+      <c r="B71" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="C71" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="E71" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="F71" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="G71" s="31"/>
+      <c r="H71" s="31"/>
+      <c r="I71" s="31"/>
+      <c r="J71" s="31"/>
+      <c r="K71" s="31"/>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A72" s="17">
-        <v>9</v>
-      </c>
-      <c r="B72" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="C72" s="19"/>
-      <c r="D72" s="19"/>
-      <c r="E72" s="19"/>
-      <c r="F72" s="19"/>
-      <c r="G72" s="19"/>
+      <c r="A72" s="17"/>
+      <c r="B72" s="18" t="str">
+        <f>B61</f>
+        <v>-for intake 1 cover</v>
+      </c>
+      <c r="C72" s="19">
+        <f>TRUNC((D73)/0.15,0)+1</f>
+        <v>12</v>
+      </c>
+      <c r="D72" s="20">
+        <f>Sheet1!G10-0.1</f>
+        <v>1.7</v>
+      </c>
+      <c r="E72" s="20">
+        <f t="shared" ref="E72:E84" si="2">10*10/162</f>
+        <v>0.61728395061728392</v>
+      </c>
+      <c r="F72" s="20">
+        <f t="shared" ref="F72:F84" si="3">PRODUCT(C72:E72)</f>
+        <v>12.592592592592592</v>
+      </c>
+      <c r="G72" s="20">
+        <f t="shared" ref="G72:G84" si="4">F72</f>
+        <v>12.592592592592592</v>
+      </c>
       <c r="H72" s="19"/>
       <c r="I72" s="19"/>
       <c r="J72" s="19"/>
@@ -2823,25 +2868,26 @@
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="17"/>
-      <c r="B73" s="18" t="str">
-        <f>B62</f>
-        <v>-for intake 1 cover</v>
-      </c>
+      <c r="B73" s="18"/>
       <c r="C73" s="19">
-        <v>1</v>
+        <f>TRUNC((D72)/0.15,0)+1</f>
+        <v>12</v>
       </c>
       <c r="D73" s="20">
-        <v>1.8</v>
+        <f>Sheet1!H10-0.1</f>
+        <v>1.7</v>
       </c>
       <c r="E73" s="20">
-        <v>1.8</v>
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
       </c>
       <c r="F73" s="20">
-        <v>0.1</v>
+        <f t="shared" si="3"/>
+        <v>12.592592592592592</v>
       </c>
       <c r="G73" s="20">
-        <f t="shared" ref="G73:G80" si="1">PRODUCT(C73:F73)</f>
-        <v>0.32400000000000007</v>
+        <f t="shared" si="4"/>
+        <v>12.592592592592592</v>
       </c>
       <c r="H73" s="19"/>
       <c r="I73" s="19"/>
@@ -2851,24 +2897,28 @@
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="17"/>
       <c r="B74" s="18" t="str">
-        <f>B18</f>
+        <f>B62</f>
         <v>-for intake 2</v>
       </c>
       <c r="C74" s="19">
-        <v>1</v>
+        <f>TRUNC((Sheet1!G11-0.1)/0.15,0)+1</f>
+        <v>13</v>
       </c>
       <c r="D74" s="20">
-        <v>2</v>
+        <f>(Sheet1!H11-Sheet1!J11)+(Sheet1!I11-0.05+Sheet1!J11/2)*2</f>
+        <v>4.3</v>
       </c>
       <c r="E74" s="20">
-        <v>2</v>
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
       </c>
       <c r="F74" s="20">
-        <v>0.1</v>
+        <f t="shared" si="3"/>
+        <v>34.506172839506171</v>
       </c>
       <c r="G74" s="20">
-        <f t="shared" si="1"/>
-        <v>0.4</v>
+        <f t="shared" si="4"/>
+        <v>34.506172839506171</v>
       </c>
       <c r="H74" s="19"/>
       <c r="I74" s="19"/>
@@ -2877,24 +2927,26 @@
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="17"/>
-      <c r="B75" s="18" t="s">
-        <v>93</v>
-      </c>
+      <c r="B75" s="18"/>
       <c r="C75" s="19">
-        <v>2</v>
+        <f>TRUNC((Sheet1!H11-0.1)/0.15,0)+1</f>
+        <v>13</v>
       </c>
       <c r="D75" s="20">
-        <v>2</v>
+        <f>(Sheet1!G11-Sheet1!J11)+(Sheet1!I11-0.05+Sheet1!J11/2)*2</f>
+        <v>4.3</v>
       </c>
       <c r="E75" s="20">
-        <v>0.1</v>
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
       </c>
       <c r="F75" s="20">
-        <v>1.2</v>
+        <f t="shared" si="3"/>
+        <v>34.506172839506171</v>
       </c>
       <c r="G75" s="20">
-        <f t="shared" si="1"/>
-        <v>0.48</v>
+        <f t="shared" si="4"/>
+        <v>34.506172839506171</v>
       </c>
       <c r="H75" s="19"/>
       <c r="I75" s="19"/>
@@ -2904,23 +2956,27 @@
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="17"/>
       <c r="B76" s="18" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="C76" s="19">
-        <v>2</v>
+        <f>2*(TRUNC((Sheet1!I11+Sheet1!J11-0.05-0.05)/0.15,0)+1)</f>
+        <v>18</v>
       </c>
       <c r="D76" s="20">
-        <v>1.7999999999999998</v>
+        <f>(Sheet1!G11-0.05-0.05)*4</f>
+        <v>7.6</v>
       </c>
       <c r="E76" s="20">
-        <v>0.1</v>
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
       </c>
       <c r="F76" s="20">
-        <v>1.2</v>
+        <f t="shared" si="3"/>
+        <v>84.444444444444429</v>
       </c>
       <c r="G76" s="20">
-        <f t="shared" si="1"/>
-        <v>0.432</v>
+        <f t="shared" si="4"/>
+        <v>84.444444444444429</v>
       </c>
       <c r="H76" s="19"/>
       <c r="I76" s="19"/>
@@ -2934,20 +2990,24 @@
         <v>-for intake 2 cover</v>
       </c>
       <c r="C77" s="19">
-        <v>1</v>
+        <f>TRUNC((D78)/0.15,0)+1</f>
+        <v>13</v>
       </c>
       <c r="D77" s="20">
-        <v>2</v>
+        <f>Sheet1!G11-0.1</f>
+        <v>1.9</v>
       </c>
       <c r="E77" s="20">
-        <v>2</v>
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
       </c>
       <c r="F77" s="20">
-        <v>0.1</v>
+        <f t="shared" si="3"/>
+        <v>15.246913580246913</v>
       </c>
       <c r="G77" s="20">
-        <f t="shared" si="1"/>
-        <v>0.4</v>
+        <f t="shared" si="4"/>
+        <v>15.246913580246913</v>
       </c>
       <c r="H77" s="19"/>
       <c r="I77" s="19"/>
@@ -2956,27 +3016,26 @@
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="17"/>
-      <c r="B78" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="C78" s="21">
-        <f>C27</f>
-        <v>0.5</v>
+      <c r="B78" s="18"/>
+      <c r="C78" s="19">
+        <f>TRUNC((D77)/0.15,0)+1</f>
+        <v>13</v>
       </c>
       <c r="D78" s="20">
-        <f>D27</f>
-        <v>21.335000000000001</v>
+        <f>Sheet1!H11-0.1</f>
+        <v>1.9</v>
       </c>
       <c r="E78" s="20">
-        <f>E27</f>
-        <v>0.54999999999999993</v>
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
       </c>
       <c r="F78" s="20">
-        <v>0.1</v>
+        <f t="shared" si="3"/>
+        <v>15.246913580246913</v>
       </c>
       <c r="G78" s="20">
-        <f t="shared" si="1"/>
-        <v>0.58671249999999997</v>
+        <f t="shared" si="4"/>
+        <v>15.246913580246913</v>
       </c>
       <c r="H78" s="19"/>
       <c r="I78" s="19"/>
@@ -2985,24 +3044,29 @@
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="17"/>
-      <c r="B79" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="C79" s="21">
-        <v>2</v>
+      <c r="B79" s="18" t="str">
+        <f>B26</f>
+        <v>-for kulo</v>
+      </c>
+      <c r="C79" s="19">
+        <f>TRUNC((Sheet1!K10-0.1)/0.15,0)+1</f>
+        <v>142</v>
       </c>
       <c r="D79" s="20">
-        <v>21.34</v>
+        <f>(Sheet1!L10-0.1)+(Sheet1!M10-0.05+Sheet1!N10/2)*2</f>
+        <v>1.35</v>
       </c>
       <c r="E79" s="20">
-        <v>0.1</v>
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
       </c>
       <c r="F79" s="20">
-        <v>0.45</v>
+        <f t="shared" si="3"/>
+        <v>118.33333333333334</v>
       </c>
       <c r="G79" s="20">
-        <f t="shared" si="1"/>
-        <v>1.9205999999999999</v>
+        <f t="shared" si="4"/>
+        <v>118.33333333333334</v>
       </c>
       <c r="H79" s="19"/>
       <c r="I79" s="19"/>
@@ -3012,1049 +3076,543 @@
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="17"/>
       <c r="B80" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="C80" s="21">
-        <v>1</v>
+        <v>75</v>
+      </c>
+      <c r="C80" s="19">
+        <f>(TRUNC((Sheet1!L10-Sheet1!N10)/0.15,0)+1)+2*(TRUNC((Sheet1!M10/0.15),0)+1)</f>
+        <v>12</v>
       </c>
       <c r="D80" s="20">
-        <v>21.34</v>
+        <f>Sheet1!K10</f>
+        <v>21.334958854007922</v>
       </c>
       <c r="E80" s="20">
-        <v>0.54999999999999993</v>
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
       </c>
       <c r="F80" s="20">
-        <v>0.1</v>
+        <f t="shared" si="3"/>
+        <v>158.03673225191054</v>
       </c>
       <c r="G80" s="20">
-        <f t="shared" si="1"/>
-        <v>1.1737</v>
+        <f t="shared" si="4"/>
+        <v>158.03673225191054</v>
       </c>
       <c r="H80" s="19"/>
       <c r="I80" s="19"/>
       <c r="J80" s="19"/>
       <c r="K80" s="19"/>
     </row>
-    <row r="81" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="22"/>
-      <c r="B81" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C81" s="24"/>
-      <c r="D81" s="1"/>
-      <c r="E81" s="25"/>
-      <c r="F81" s="25"/>
-      <c r="G81" s="2">
-        <f>SUM(G73:G80)</f>
-        <v>5.7170125000000001</v>
-      </c>
-      <c r="H81" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="I81" s="2">
-        <v>14337.7</v>
-      </c>
-      <c r="J81" s="27">
-        <f>G81*I81</f>
-        <v>81968.810121250004</v>
-      </c>
-      <c r="K81" s="25"/>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A81" s="17"/>
+      <c r="B81" s="18" t="str">
+        <f>B68</f>
+        <v>-for shear wall cover slab</v>
+      </c>
+      <c r="C81" s="19">
+        <f>C57*(TRUNC((D82-0.1)/0.15,0)+1)</f>
+        <v>140</v>
+      </c>
+      <c r="D81" s="20">
+        <f>Sheet1!L10</f>
+        <v>0.54999999999999993</v>
+      </c>
+      <c r="E81" s="20">
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
+      </c>
+      <c r="F81" s="20">
+        <f t="shared" si="3"/>
+        <v>47.530864197530853</v>
+      </c>
+      <c r="G81" s="20">
+        <f t="shared" si="4"/>
+        <v>47.530864197530853</v>
+      </c>
+      <c r="H81" s="19"/>
+      <c r="I81" s="19"/>
+      <c r="J81" s="19"/>
+      <c r="K81" s="19"/>
+    </row>
+    <row r="82" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A82" s="17"/>
-      <c r="B82" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C82" s="19"/>
-      <c r="D82" s="19"/>
-      <c r="E82" s="19"/>
-      <c r="F82" s="19"/>
-      <c r="G82" s="19"/>
+      <c r="B82" s="18"/>
+      <c r="C82" s="19">
+        <f>C57*(TRUNC((D81-0.1)/0.15,0)+1)</f>
+        <v>140</v>
+      </c>
+      <c r="D82" s="20">
+        <v>0.6</v>
+      </c>
+      <c r="E82" s="20">
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
+      </c>
+      <c r="F82" s="20">
+        <f t="shared" si="3"/>
+        <v>51.851851851851848</v>
+      </c>
+      <c r="G82" s="20">
+        <f t="shared" si="4"/>
+        <v>51.851851851851848</v>
+      </c>
       <c r="H82" s="19"/>
       <c r="I82" s="19"/>
-      <c r="J82" s="27">
-        <f>0.13*G81*5120</f>
-        <v>3805.24352</v>
-      </c>
+      <c r="J82" s="19"/>
       <c r="K82" s="19"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A83" s="17"/>
       <c r="B83" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="C83" s="19"/>
-      <c r="D83" s="19"/>
-      <c r="E83" s="19"/>
-      <c r="F83" s="19"/>
-      <c r="G83" s="19"/>
+        <v>83</v>
+      </c>
+      <c r="C83" s="19">
+        <f>TRUNC((D84)/0.15,0)+1</f>
+        <v>12</v>
+      </c>
+      <c r="D83" s="20">
+        <f>1.5-0.1</f>
+        <v>1.4</v>
+      </c>
+      <c r="E83" s="20">
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
+      </c>
+      <c r="F83" s="20">
+        <f t="shared" si="3"/>
+        <v>10.370370370370368</v>
+      </c>
+      <c r="G83" s="20">
+        <f t="shared" si="4"/>
+        <v>10.370370370370368</v>
+      </c>
       <c r="H83" s="19"/>
       <c r="I83" s="19"/>
-      <c r="J83" s="27">
-        <f>0.13*G81*1349.75</f>
-        <v>1003.1498908437501</v>
-      </c>
+      <c r="J83" s="19"/>
       <c r="K83" s="19"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A84" s="17"/>
-      <c r="B84" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="C84" s="19"/>
-      <c r="D84" s="19"/>
-      <c r="E84" s="19"/>
-      <c r="F84" s="19"/>
-      <c r="G84" s="19"/>
+      <c r="B84" s="18"/>
+      <c r="C84" s="19">
+        <f>TRUNC((D83)/0.15,0)+1</f>
+        <v>10</v>
+      </c>
+      <c r="D84" s="20">
+        <f>1.8-0.1</f>
+        <v>1.7</v>
+      </c>
+      <c r="E84" s="20">
+        <f t="shared" si="2"/>
+        <v>0.61728395061728392</v>
+      </c>
+      <c r="F84" s="20">
+        <f t="shared" si="3"/>
+        <v>10.493827160493826</v>
+      </c>
+      <c r="G84" s="20">
+        <f t="shared" si="4"/>
+        <v>10.493827160493826</v>
+      </c>
       <c r="H84" s="19"/>
       <c r="I84" s="19"/>
-      <c r="J84" s="27">
-        <f>0.13*G81*(972.17+1910.82)</f>
-        <v>2142.6716827587497</v>
-      </c>
+      <c r="J84" s="19"/>
       <c r="K84" s="19"/>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A85" s="17"/>
-      <c r="B85" s="19"/>
-      <c r="C85" s="19"/>
-      <c r="D85" s="19"/>
-      <c r="E85" s="19"/>
-      <c r="F85" s="19"/>
-      <c r="G85" s="19"/>
-      <c r="H85" s="19"/>
-      <c r="I85" s="19"/>
-      <c r="J85" s="19"/>
-      <c r="K85" s="19"/>
-    </row>
-    <row r="86" spans="1:11" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A86" s="17">
-        <v>10</v>
-      </c>
-      <c r="B86" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="C86" s="31" t="s">
-        <v>7</v>
-      </c>
-      <c r="D86" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="E86" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="F86" s="32" t="s">
-        <v>57</v>
-      </c>
-      <c r="G86" s="31"/>
-      <c r="H86" s="31"/>
-      <c r="I86" s="31"/>
-      <c r="J86" s="31"/>
-      <c r="K86" s="31"/>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A87" s="17"/>
-      <c r="B87" s="18" t="str">
-        <f>B73</f>
-        <v>-for intake 1 cover</v>
-      </c>
-      <c r="C87" s="19">
-        <f>TRUNC((D88)/0.15,0)+1</f>
-        <v>12</v>
-      </c>
-      <c r="D87" s="20">
-        <f>Sheet1!G10-0.1</f>
-        <v>1.7</v>
-      </c>
-      <c r="E87" s="20">
-        <f t="shared" ref="E87:E99" si="2">10*10/162</f>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F87" s="20">
-        <f t="shared" ref="F87:F99" si="3">PRODUCT(C87:E87)</f>
-        <v>12.592592592592592</v>
-      </c>
-      <c r="G87" s="20">
-        <f t="shared" ref="G87:G99" si="4">F87</f>
-        <v>12.592592592592592</v>
-      </c>
-      <c r="H87" s="19"/>
-      <c r="I87" s="19"/>
-      <c r="J87" s="19"/>
-      <c r="K87" s="19"/>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A88" s="17"/>
-      <c r="B88" s="18"/>
-      <c r="C88" s="19">
-        <f>TRUNC((D87)/0.15,0)+1</f>
-        <v>12</v>
-      </c>
-      <c r="D88" s="20">
-        <f>Sheet1!H10-0.1</f>
-        <v>1.7</v>
-      </c>
-      <c r="E88" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F88" s="20">
-        <f t="shared" si="3"/>
-        <v>12.592592592592592</v>
-      </c>
-      <c r="G88" s="20">
-        <f t="shared" si="4"/>
-        <v>12.592592592592592</v>
-      </c>
+    <row r="85" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="22"/>
+      <c r="B85" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C85" s="24"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="25"/>
+      <c r="F85" s="25"/>
+      <c r="G85" s="2">
+        <f>SUM(G72:G84)</f>
+        <v>605.75278163462656</v>
+      </c>
+      <c r="H85" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="I85" s="2">
+        <f>1.15*9831.6/100</f>
+        <v>113.0634</v>
+      </c>
+      <c r="J85" s="27">
+        <f>G85*I85</f>
+        <v>68488.46905106843</v>
+      </c>
+      <c r="K85" s="25"/>
+    </row>
+    <row r="86" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A86" s="17"/>
+      <c r="B86" s="19"/>
+      <c r="C86" s="19"/>
+      <c r="D86" s="19"/>
+      <c r="E86" s="19"/>
+      <c r="F86" s="19"/>
+      <c r="G86" s="19"/>
+      <c r="H86" s="19"/>
+      <c r="I86" s="19"/>
+      <c r="J86" s="19"/>
+      <c r="K86" s="19"/>
+    </row>
+    <row r="87" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A87" s="7"/>
+      <c r="B87" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C87" s="7"/>
+      <c r="D87" s="9"/>
+      <c r="E87" s="9"/>
+      <c r="F87" s="9"/>
+      <c r="G87" s="9"/>
+      <c r="H87" s="7"/>
+      <c r="I87" s="9"/>
+      <c r="J87" s="9"/>
+      <c r="K87" s="10"/>
+    </row>
+    <row r="88" spans="1:27" ht="33" x14ac:dyDescent="0.25">
+      <c r="A88" s="17">
+        <v>11</v>
+      </c>
+      <c r="B88" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C88" s="19"/>
+      <c r="D88" s="19"/>
+      <c r="E88" s="19"/>
+      <c r="F88" s="19"/>
+      <c r="G88" s="19"/>
       <c r="H88" s="19"/>
       <c r="I88" s="19"/>
-      <c r="J88" s="19"/>
+      <c r="J88" s="27"/>
       <c r="K88" s="19"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A89" s="17"/>
-      <c r="B89" s="18" t="str">
-        <f>B74</f>
-        <v>-for intake 2</v>
+      <c r="B89" s="18" t="s">
+        <v>34</v>
       </c>
       <c r="C89" s="19">
-        <f>TRUNC((Sheet1!G11-0.1)/0.15,0)+1</f>
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D89" s="20">
-        <f>(Sheet1!H11-Sheet1!J11)+(Sheet1!I11-0.05+Sheet1!J11/2)*2</f>
-        <v>4.3</v>
-      </c>
-      <c r="E89" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F89" s="20">
-        <f t="shared" si="3"/>
-        <v>34.506172839506171</v>
+        <f>D97-TRUNC(0.25*D97,0)</f>
+        <v>188</v>
+      </c>
+      <c r="E89" s="19">
+        <v>0.3</v>
+      </c>
+      <c r="F89" s="19">
+        <v>0.45</v>
       </c>
       <c r="G89" s="20">
-        <f t="shared" si="4"/>
-        <v>34.506172839506171</v>
+        <f>PRODUCT(C89:F89)</f>
+        <v>25.38</v>
       </c>
       <c r="H89" s="19"/>
       <c r="I89" s="19"/>
-      <c r="J89" s="19"/>
+      <c r="J89" s="27"/>
       <c r="K89" s="19"/>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A90" s="17"/>
-      <c r="B90" s="18"/>
-      <c r="C90" s="19">
-        <f>TRUNC((Sheet1!H11-0.1)/0.15,0)+1</f>
-        <v>13</v>
-      </c>
-      <c r="D90" s="20">
-        <f>(Sheet1!G11-Sheet1!J11)+(Sheet1!I11-0.05+Sheet1!J11/2)*2</f>
-        <v>4.3</v>
-      </c>
-      <c r="E90" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F90" s="20">
-        <f t="shared" si="3"/>
-        <v>34.506172839506171</v>
-      </c>
-      <c r="G90" s="20">
-        <f t="shared" si="4"/>
-        <v>34.506172839506171</v>
-      </c>
-      <c r="H90" s="19"/>
-      <c r="I90" s="19"/>
-      <c r="J90" s="19"/>
-      <c r="K90" s="19"/>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="AA89" s="11"/>
+    </row>
+    <row r="90" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="22"/>
+      <c r="B90" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="C90" s="24"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="25"/>
+      <c r="F90" s="25"/>
+      <c r="G90" s="30">
+        <f>SUM(G89:G89)</f>
+        <v>25.38</v>
+      </c>
+      <c r="H90" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="I90" s="2">
+        <f>1.15*963.05</f>
+        <v>1107.5074999999999</v>
+      </c>
+      <c r="J90" s="30">
+        <f>G90*I90</f>
+        <v>28108.540349999996</v>
+      </c>
+      <c r="K90" s="25"/>
+      <c r="AA90" s="4"/>
+    </row>
+    <row r="91" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A91" s="17"/>
-      <c r="B91" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="C91" s="19">
-        <f>2*(TRUNC((Sheet1!I11+Sheet1!J11-0.05-0.05)/0.15,0)+1)</f>
-        <v>18</v>
-      </c>
-      <c r="D91" s="20">
-        <f>(Sheet1!G11-0.05-0.05)*4</f>
-        <v>7.6</v>
-      </c>
-      <c r="E91" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F91" s="20">
-        <f t="shared" si="3"/>
-        <v>84.444444444444429</v>
-      </c>
-      <c r="G91" s="20">
-        <f t="shared" si="4"/>
-        <v>84.444444444444429</v>
-      </c>
+      <c r="B91" s="18"/>
+      <c r="C91" s="19"/>
+      <c r="D91" s="19"/>
+      <c r="E91" s="19"/>
+      <c r="F91" s="19"/>
+      <c r="G91" s="19"/>
       <c r="H91" s="19"/>
       <c r="I91" s="19"/>
-      <c r="J91" s="19"/>
+      <c r="J91" s="27"/>
       <c r="K91" s="19"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A92" s="17"/>
-      <c r="B92" s="18" t="str">
-        <f>B77</f>
-        <v>-for intake 2 cover</v>
-      </c>
-      <c r="C92" s="19">
-        <f>TRUNC((D93)/0.15,0)+1</f>
-        <v>13</v>
-      </c>
-      <c r="D92" s="20">
-        <f>Sheet1!G11-0.1</f>
-        <v>1.9</v>
-      </c>
-      <c r="E92" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F92" s="20">
-        <f t="shared" si="3"/>
-        <v>15.246913580246913</v>
-      </c>
-      <c r="G92" s="20">
-        <f t="shared" si="4"/>
-        <v>15.246913580246913</v>
-      </c>
+    <row r="92" spans="1:27" ht="30" x14ac:dyDescent="0.25">
+      <c r="A92" s="17">
+        <v>12</v>
+      </c>
+      <c r="B92" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C92" s="19"/>
+      <c r="D92" s="19"/>
+      <c r="E92" s="19"/>
+      <c r="F92" s="19"/>
+      <c r="G92" s="19"/>
       <c r="H92" s="19"/>
       <c r="I92" s="19"/>
       <c r="J92" s="19"/>
       <c r="K92" s="19"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A93" s="17"/>
-      <c r="B93" s="18"/>
+      <c r="B93" s="18" t="s">
+        <v>30</v>
+      </c>
       <c r="C93" s="19">
-        <f>TRUNC((D92)/0.15,0)+1</f>
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D93" s="20">
-        <f>Sheet1!H11-0.1</f>
-        <v>1.9</v>
-      </c>
-      <c r="E93" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F93" s="20">
-        <f t="shared" si="3"/>
-        <v>15.246913580246913</v>
-      </c>
+        <f>D97</f>
+        <v>250</v>
+      </c>
+      <c r="E93" s="19"/>
+      <c r="F93" s="19"/>
       <c r="G93" s="20">
-        <f t="shared" si="4"/>
-        <v>15.246913580246913</v>
+        <f>PRODUCT(C93:F93)</f>
+        <v>250</v>
       </c>
       <c r="H93" s="19"/>
       <c r="I93" s="19"/>
-      <c r="J93" s="19"/>
+      <c r="J93" s="27"/>
       <c r="K93" s="19"/>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A94" s="17"/>
-      <c r="B94" s="18" t="str">
-        <f>B27</f>
-        <v>-for kulo</v>
-      </c>
-      <c r="C94" s="19">
-        <f>TRUNC((Sheet1!K10-0.1)/0.15,0)+1</f>
-        <v>142</v>
-      </c>
-      <c r="D94" s="20">
-        <f>(Sheet1!L10-0.1)+(Sheet1!M10-0.05+Sheet1!N10/2)*2</f>
-        <v>1.35</v>
-      </c>
-      <c r="E94" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F94" s="20">
-        <f t="shared" si="3"/>
-        <v>118.33333333333334</v>
-      </c>
-      <c r="G94" s="20">
-        <f t="shared" si="4"/>
-        <v>118.33333333333334</v>
-      </c>
-      <c r="H94" s="19"/>
-      <c r="I94" s="19"/>
-      <c r="J94" s="19"/>
-      <c r="K94" s="19"/>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="AA93" s="11"/>
+    </row>
+    <row r="94" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="22"/>
+      <c r="B94" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="C94" s="24"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="25"/>
+      <c r="F94" s="25"/>
+      <c r="G94" s="30">
+        <f>SUM(G93:G93)</f>
+        <v>250</v>
+      </c>
+      <c r="H94" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="I94" s="2">
+        <f>1.15*4308.15/1000</f>
+        <v>4.9543724999999998</v>
+      </c>
+      <c r="J94" s="30">
+        <f>G94*I94</f>
+        <v>1238.5931249999999</v>
+      </c>
+      <c r="K94" s="25"/>
+      <c r="AA94" s="4"/>
+    </row>
+    <row r="95" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A95" s="17"/>
-      <c r="B95" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="C95" s="19">
-        <f>(TRUNC((Sheet1!L10-Sheet1!N10)/0.15,0)+1)+2*(TRUNC((Sheet1!M10/0.15),0)+1)</f>
-        <v>12</v>
-      </c>
-      <c r="D95" s="20">
-        <f>Sheet1!K10</f>
-        <v>21.334958854007922</v>
-      </c>
-      <c r="E95" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F95" s="20">
-        <f t="shared" si="3"/>
-        <v>158.03673225191054</v>
-      </c>
-      <c r="G95" s="20">
-        <f t="shared" si="4"/>
-        <v>158.03673225191054</v>
-      </c>
+      <c r="B95" s="13"/>
+      <c r="C95" s="19"/>
+      <c r="D95" s="19"/>
+      <c r="E95" s="19"/>
+      <c r="F95" s="19"/>
+      <c r="G95" s="19"/>
       <c r="H95" s="19"/>
       <c r="I95" s="19"/>
       <c r="J95" s="19"/>
       <c r="K95" s="19"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A96" s="17"/>
-      <c r="B96" s="18" t="str">
-        <f>B80</f>
-        <v>-for shear wall cover slab</v>
-      </c>
-      <c r="C96" s="19">
-        <f>C67*(TRUNC((D97-0.1)/0.15,0)+1)</f>
-        <v>140</v>
-      </c>
-      <c r="D96" s="20">
-        <f>Sheet1!L10</f>
-        <v>0.54999999999999993</v>
-      </c>
-      <c r="E96" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F96" s="20">
-        <f t="shared" si="3"/>
-        <v>47.530864197530853</v>
-      </c>
-      <c r="G96" s="20">
-        <f t="shared" si="4"/>
-        <v>47.530864197530853</v>
-      </c>
+    <row r="96" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+      <c r="A96" s="17">
+        <v>13</v>
+      </c>
+      <c r="B96" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C96" s="19"/>
+      <c r="D96" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E96" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="F96" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G96" s="19"/>
       <c r="H96" s="19"/>
       <c r="I96" s="19"/>
-      <c r="J96" s="19"/>
+      <c r="J96" s="27"/>
       <c r="K96" s="19"/>
-    </row>
-    <row r="97" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AA96" s="11"/>
+    </row>
+    <row r="97" spans="1:27" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A97" s="17"/>
-      <c r="B97" s="18"/>
-      <c r="C97" s="19">
-        <f>C67*(TRUNC((D96-0.1)/0.15,0)+1)</f>
-        <v>140</v>
-      </c>
-      <c r="D97" s="20">
-        <v>0.6</v>
-      </c>
-      <c r="E97" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F97" s="20">
-        <f t="shared" si="3"/>
-        <v>51.851851851851848</v>
-      </c>
-      <c r="G97" s="20">
-        <f t="shared" si="4"/>
-        <v>51.851851851851848</v>
-      </c>
-      <c r="H97" s="19"/>
-      <c r="I97" s="19"/>
-      <c r="J97" s="19"/>
-      <c r="K97" s="19"/>
-    </row>
-    <row r="98" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A98" s="17"/>
-      <c r="B98" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="C98" s="19">
-        <f>TRUNC((D99)/0.15,0)+1</f>
-        <v>12</v>
-      </c>
-      <c r="D98" s="20">
-        <f>1.5-0.1</f>
-        <v>1.4</v>
-      </c>
-      <c r="E98" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F98" s="20">
-        <f t="shared" si="3"/>
-        <v>10.370370370370368</v>
-      </c>
-      <c r="G98" s="20">
-        <f t="shared" si="4"/>
-        <v>10.370370370370368</v>
-      </c>
-      <c r="H98" s="19"/>
-      <c r="I98" s="19"/>
-      <c r="J98" s="19"/>
-      <c r="K98" s="19"/>
+      <c r="B97" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="C97" s="31">
+        <v>1</v>
+      </c>
+      <c r="D97" s="36">
+        <v>250</v>
+      </c>
+      <c r="E97" s="31">
+        <v>0.20799999999999999</v>
+      </c>
+      <c r="F97" s="31">
+        <f>C97*D97*E97</f>
+        <v>52</v>
+      </c>
+      <c r="G97" s="36">
+        <f>F97</f>
+        <v>52</v>
+      </c>
+      <c r="H97" s="31"/>
+      <c r="I97" s="31"/>
+      <c r="J97" s="26"/>
+      <c r="K97" s="31"/>
+      <c r="AA97" s="4"/>
+    </row>
+    <row r="98" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="22"/>
+      <c r="B98" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C98" s="24"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="25"/>
+      <c r="F98" s="25"/>
+      <c r="G98" s="2">
+        <f>SUM(G97:G97)</f>
+        <v>52</v>
+      </c>
+      <c r="H98" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="I98" s="2">
+        <v>287</v>
+      </c>
+      <c r="J98" s="27">
+        <f>G98*I98</f>
+        <v>14924</v>
+      </c>
+      <c r="K98" s="25"/>
     </row>
     <row r="99" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A99" s="17"/>
-      <c r="B99" s="18"/>
-      <c r="C99" s="19">
-        <f>TRUNC((D98)/0.15,0)+1</f>
-        <v>10</v>
-      </c>
-      <c r="D99" s="20">
-        <f>1.8-0.1</f>
-        <v>1.7</v>
-      </c>
-      <c r="E99" s="20">
-        <f t="shared" si="2"/>
-        <v>0.61728395061728392</v>
-      </c>
-      <c r="F99" s="20">
-        <f t="shared" si="3"/>
-        <v>10.493827160493826</v>
-      </c>
-      <c r="G99" s="20">
-        <f t="shared" si="4"/>
-        <v>10.493827160493826</v>
-      </c>
+      <c r="B99" s="19"/>
+      <c r="C99" s="19"/>
+      <c r="D99" s="19"/>
+      <c r="E99" s="19"/>
+      <c r="F99" s="19"/>
+      <c r="G99" s="19"/>
       <c r="H99" s="19"/>
       <c r="I99" s="19"/>
       <c r="J99" s="19"/>
       <c r="K99" s="19"/>
     </row>
     <row r="100" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="22"/>
-      <c r="B100" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C100" s="24"/>
+      <c r="A100" s="22">
+        <v>14</v>
+      </c>
+      <c r="B100" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="C100" s="24">
+        <v>1</v>
+      </c>
       <c r="D100" s="1"/>
       <c r="E100" s="25"/>
       <c r="F100" s="25"/>
-      <c r="G100" s="2">
-        <f>SUM(G87:G99)</f>
-        <v>605.75278163462656</v>
+      <c r="G100" s="26">
+        <f>PRODUCT(C100:F100)</f>
+        <v>1</v>
       </c>
       <c r="H100" s="26" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="I100" s="2">
-        <f>9831.6/100</f>
-        <v>98.316000000000003</v>
-      </c>
-      <c r="J100" s="27">
+        <v>500</v>
+      </c>
+      <c r="J100" s="26">
         <f>G100*I100</f>
-        <v>59555.190479189943</v>
+        <v>500</v>
       </c>
       <c r="K100" s="25"/>
     </row>
     <row r="101" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A101" s="17"/>
-      <c r="B101" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="C101" s="19"/>
-      <c r="D101" s="19"/>
-      <c r="E101" s="19"/>
-      <c r="F101" s="19"/>
-      <c r="G101" s="19"/>
-      <c r="H101" s="19"/>
-      <c r="I101" s="19"/>
-      <c r="J101" s="27">
-        <f>0.13*G100*9450/100</f>
-        <v>7441.6729223813873</v>
-      </c>
-      <c r="K101" s="19"/>
+      <c r="A101" s="22"/>
+      <c r="B101" s="38"/>
+      <c r="C101" s="24"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="25"/>
+      <c r="F101" s="25"/>
+      <c r="G101" s="2"/>
+      <c r="H101" s="26"/>
+      <c r="I101" s="2"/>
+      <c r="J101" s="27"/>
+      <c r="K101" s="25"/>
     </row>
     <row r="102" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A102" s="17"/>
-      <c r="B102" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="C102" s="19"/>
-      <c r="D102" s="19"/>
-      <c r="E102" s="19"/>
-      <c r="F102" s="19"/>
-      <c r="G102" s="19"/>
-      <c r="H102" s="19"/>
-      <c r="I102" s="19"/>
+      <c r="A102" s="39"/>
+      <c r="B102" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="C102" s="41"/>
+      <c r="D102" s="42"/>
+      <c r="E102" s="42"/>
+      <c r="F102" s="42"/>
+      <c r="G102" s="27"/>
+      <c r="H102" s="27"/>
+      <c r="I102" s="27"/>
       <c r="J102" s="27">
-        <f>0.13*G100*120/100</f>
-        <v>94.497433935001737</v>
-      </c>
-      <c r="K102" s="19"/>
+        <f>SUM(J10:J100)</f>
+        <v>397458.98805984226</v>
+      </c>
+      <c r="K102" s="43"/>
     </row>
     <row r="103" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A103" s="17"/>
-      <c r="B103" s="19"/>
-      <c r="C103" s="19"/>
-      <c r="D103" s="19"/>
-      <c r="E103" s="19"/>
-      <c r="F103" s="19"/>
-      <c r="G103" s="19"/>
-      <c r="H103" s="19"/>
-      <c r="I103" s="19"/>
-      <c r="J103" s="19"/>
-      <c r="K103" s="19"/>
-    </row>
-    <row r="104" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A104" s="7"/>
-      <c r="B104" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C104" s="7"/>
-      <c r="D104" s="9"/>
-      <c r="E104" s="9"/>
-      <c r="F104" s="9"/>
-      <c r="G104" s="9"/>
-      <c r="H104" s="7"/>
-      <c r="I104" s="9"/>
-      <c r="J104" s="9"/>
-      <c r="K104" s="10"/>
-    </row>
-    <row r="105" spans="1:27" ht="33" x14ac:dyDescent="0.25">
-      <c r="A105" s="17">
-        <v>11</v>
-      </c>
-      <c r="B105" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C105" s="19"/>
-      <c r="D105" s="19"/>
-      <c r="E105" s="19"/>
-      <c r="F105" s="19"/>
-      <c r="G105" s="19"/>
-      <c r="H105" s="19"/>
-      <c r="I105" s="19"/>
-      <c r="J105" s="27"/>
-      <c r="K105" s="19"/>
-    </row>
-    <row r="106" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A106" s="17"/>
-      <c r="B106" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C106" s="19">
-        <v>1</v>
-      </c>
-      <c r="D106" s="20">
-        <f>D114-TRUNC(0.25*D114,0)</f>
-        <v>188</v>
-      </c>
-      <c r="E106" s="19">
-        <v>0.3</v>
-      </c>
-      <c r="F106" s="19">
-        <v>0.45</v>
-      </c>
-      <c r="G106" s="20">
-        <f>PRODUCT(C106:F106)</f>
-        <v>25.38</v>
-      </c>
-      <c r="H106" s="19"/>
-      <c r="I106" s="19"/>
-      <c r="J106" s="27"/>
-      <c r="K106" s="19"/>
-      <c r="AA106" s="11"/>
-    </row>
-    <row r="107" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="22"/>
-      <c r="B107" s="33" t="s">
-        <v>28</v>
-      </c>
-      <c r="C107" s="24"/>
-      <c r="D107" s="1"/>
-      <c r="E107" s="25"/>
-      <c r="F107" s="25"/>
-      <c r="G107" s="30">
-        <f>SUM(G106:G106)</f>
-        <v>25.38</v>
-      </c>
-      <c r="H107" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="I107" s="2">
-        <v>963.05</v>
-      </c>
-      <c r="J107" s="30">
-        <f>G107*I107</f>
-        <v>24442.208999999999</v>
-      </c>
-      <c r="K107" s="25"/>
-      <c r="AA107" s="4"/>
-    </row>
-    <row r="108" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A108" s="17"/>
-      <c r="B108" s="18"/>
-      <c r="C108" s="19"/>
-      <c r="D108" s="19"/>
-      <c r="E108" s="19"/>
-      <c r="F108" s="19"/>
-      <c r="G108" s="19"/>
-      <c r="H108" s="19"/>
-      <c r="I108" s="19"/>
-      <c r="J108" s="27"/>
-      <c r="K108" s="19"/>
-    </row>
-    <row r="109" spans="1:27" ht="30" x14ac:dyDescent="0.25">
-      <c r="A109" s="17">
-        <v>12</v>
-      </c>
-      <c r="B109" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C109" s="19"/>
-      <c r="D109" s="19"/>
-      <c r="E109" s="19"/>
-      <c r="F109" s="19"/>
-      <c r="G109" s="19"/>
-      <c r="H109" s="19"/>
-      <c r="I109" s="19"/>
-      <c r="J109" s="19"/>
-      <c r="K109" s="19"/>
-    </row>
-    <row r="110" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A110" s="17"/>
-      <c r="B110" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="C110" s="19">
-        <v>1</v>
-      </c>
-      <c r="D110" s="20">
-        <f>D114</f>
-        <v>250</v>
-      </c>
-      <c r="E110" s="19"/>
-      <c r="F110" s="19"/>
-      <c r="G110" s="20">
-        <f>PRODUCT(C110:F110)</f>
-        <v>250</v>
-      </c>
-      <c r="H110" s="19"/>
-      <c r="I110" s="19"/>
-      <c r="J110" s="27"/>
-      <c r="K110" s="19"/>
-      <c r="AA110" s="11"/>
-    </row>
-    <row r="111" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="22"/>
-      <c r="B111" s="33" t="s">
-        <v>28</v>
-      </c>
-      <c r="C111" s="24"/>
-      <c r="D111" s="1"/>
-      <c r="E111" s="25"/>
-      <c r="F111" s="25"/>
-      <c r="G111" s="30">
-        <f>SUM(G110:G110)</f>
-        <v>250</v>
-      </c>
-      <c r="H111" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="I111" s="2">
-        <f>4308.15/1000</f>
-        <v>4.3081499999999995</v>
-      </c>
-      <c r="J111" s="30">
-        <f>G111*I111</f>
-        <v>1077.0374999999999</v>
-      </c>
-      <c r="K111" s="25"/>
-      <c r="AA111" s="4"/>
-    </row>
-    <row r="112" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A112" s="17"/>
-      <c r="B112" s="13"/>
-      <c r="C112" s="19"/>
-      <c r="D112" s="19"/>
-      <c r="E112" s="19"/>
-      <c r="F112" s="19"/>
-      <c r="G112" s="19"/>
-      <c r="H112" s="19"/>
-      <c r="I112" s="19"/>
-      <c r="J112" s="19"/>
-      <c r="K112" s="19"/>
-    </row>
-    <row r="113" spans="1:27" ht="45" x14ac:dyDescent="0.25">
-      <c r="A113" s="17">
-        <v>13</v>
-      </c>
-      <c r="B113" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="C113" s="19"/>
-      <c r="D113" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E113" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="F113" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="G113" s="19"/>
-      <c r="H113" s="19"/>
-      <c r="I113" s="19"/>
-      <c r="J113" s="27"/>
-      <c r="K113" s="19"/>
-      <c r="AA113" s="11"/>
-    </row>
-    <row r="114" spans="1:27" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A114" s="17"/>
-      <c r="B114" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="C114" s="31">
-        <v>1</v>
-      </c>
-      <c r="D114" s="36">
-        <v>250</v>
-      </c>
-      <c r="E114" s="31">
-        <v>0.20799999999999999</v>
-      </c>
-      <c r="F114" s="31">
-        <f>C114*D114*E114</f>
-        <v>52</v>
-      </c>
-      <c r="G114" s="36">
-        <f>F114</f>
-        <v>52</v>
-      </c>
-      <c r="H114" s="31"/>
-      <c r="I114" s="31"/>
-      <c r="J114" s="26"/>
-      <c r="K114" s="31"/>
-      <c r="AA114" s="4"/>
-    </row>
-    <row r="115" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="22"/>
-      <c r="B115" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C115" s="24"/>
-      <c r="D115" s="1"/>
-      <c r="E115" s="25"/>
-      <c r="F115" s="25"/>
-      <c r="G115" s="2">
-        <f>SUM(G114:G114)</f>
-        <v>52</v>
-      </c>
-      <c r="H115" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="I115" s="2">
-        <v>287</v>
-      </c>
-      <c r="J115" s="27">
-        <f>G115*I115</f>
-        <v>14924</v>
-      </c>
-      <c r="K115" s="25"/>
-    </row>
-    <row r="116" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A116" s="17"/>
-      <c r="B116" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="C116" s="19"/>
-      <c r="D116" s="19"/>
-      <c r="E116" s="19"/>
-      <c r="F116" s="19"/>
-      <c r="G116" s="19"/>
-      <c r="H116" s="19"/>
-      <c r="I116" s="19"/>
-      <c r="J116" s="27">
-        <f>0.13*J115</f>
-        <v>1940.1200000000001</v>
-      </c>
-      <c r="K116" s="19"/>
-    </row>
-    <row r="117" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A117" s="17"/>
-      <c r="B117" s="19"/>
-      <c r="C117" s="19"/>
-      <c r="D117" s="19"/>
-      <c r="E117" s="19"/>
-      <c r="F117" s="19"/>
-      <c r="G117" s="19"/>
-      <c r="H117" s="19"/>
-      <c r="I117" s="19"/>
-      <c r="J117" s="19"/>
-      <c r="K117" s="19"/>
-    </row>
-    <row r="118" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="22">
-        <v>14</v>
-      </c>
-      <c r="B118" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="C118" s="24">
-        <v>1</v>
-      </c>
-      <c r="D118" s="1"/>
-      <c r="E118" s="25"/>
-      <c r="F118" s="25"/>
-      <c r="G118" s="26">
-        <f>PRODUCT(C118:F118)</f>
-        <v>1</v>
-      </c>
-      <c r="H118" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="I118" s="2">
-        <v>500</v>
-      </c>
-      <c r="J118" s="26">
-        <f>G118*I118</f>
-        <v>500</v>
-      </c>
-      <c r="K118" s="25"/>
-    </row>
-    <row r="119" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A119" s="22"/>
-      <c r="B119" s="38"/>
-      <c r="C119" s="24"/>
-      <c r="D119" s="1"/>
-      <c r="E119" s="25"/>
-      <c r="F119" s="25"/>
-      <c r="G119" s="2"/>
-      <c r="H119" s="26"/>
-      <c r="I119" s="2"/>
-      <c r="J119" s="27"/>
-      <c r="K119" s="25"/>
-    </row>
-    <row r="120" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A120" s="39"/>
-      <c r="B120" s="40" t="s">
-        <v>20</v>
-      </c>
-      <c r="C120" s="41"/>
-      <c r="D120" s="42"/>
-      <c r="E120" s="42"/>
-      <c r="F120" s="42"/>
-      <c r="G120" s="27"/>
-      <c r="H120" s="27"/>
-      <c r="I120" s="27"/>
-      <c r="J120" s="27">
-        <f>SUM(J10:J118)</f>
-        <v>375126.23303270183</v>
-      </c>
-      <c r="K120" s="43"/>
-    </row>
-    <row r="121" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="AA121" s="11"/>
-    </row>
-    <row r="122" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="44"/>
-      <c r="B122" s="31" t="s">
+      <c r="AA103" s="11"/>
+    </row>
+    <row r="104" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="44"/>
+      <c r="B104" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="C122" s="57">
-        <f>J120</f>
-        <v>375126.23303270183</v>
-      </c>
-      <c r="D122" s="58"/>
-      <c r="E122" s="36">
-        <v>100</v>
-      </c>
-      <c r="F122" s="44"/>
-      <c r="G122" s="45"/>
-      <c r="H122" s="44"/>
-      <c r="I122" s="46"/>
-      <c r="J122" s="47"/>
-      <c r="K122" s="48"/>
-      <c r="AA122" s="4"/>
-    </row>
-    <row r="123" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B123" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="C123" s="59">
-        <v>330000</v>
-      </c>
-      <c r="D123" s="60"/>
-      <c r="E123" s="36"/>
-    </row>
-    <row r="124" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B124" s="31" t="s">
-        <v>22</v>
-      </c>
-      <c r="C124" s="59">
-        <f>C123-C126-C127</f>
-        <v>313500</v>
-      </c>
-      <c r="D124" s="60"/>
-      <c r="E124" s="36">
-        <f>C124/C122*100</f>
-        <v>83.571867919104037</v>
-      </c>
-    </row>
-    <row r="125" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B125" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="C125" s="61">
-        <f>C122-C124</f>
-        <v>61626.233032701828</v>
-      </c>
-      <c r="D125" s="61"/>
-      <c r="E125" s="36">
-        <f>100-E124</f>
-        <v>16.428132080895963</v>
-      </c>
-    </row>
-    <row r="126" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B126" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="C126" s="57">
-        <f>C123*0.03</f>
-        <v>9900</v>
-      </c>
-      <c r="D126" s="58"/>
-      <c r="E126" s="36">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="127" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B127" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C127" s="57">
-        <f>C123*0.02</f>
-        <v>6600</v>
-      </c>
-      <c r="D127" s="58"/>
-      <c r="E127" s="36">
-        <v>2</v>
-      </c>
+      <c r="C104" s="49">
+        <f>J102</f>
+        <v>397458.98805984226</v>
+      </c>
+      <c r="D104" s="50"/>
+      <c r="E104" s="36"/>
+      <c r="F104" s="44"/>
+      <c r="G104" s="45"/>
+      <c r="H104" s="44"/>
+      <c r="I104" s="46"/>
+      <c r="J104" s="47"/>
+      <c r="K104" s="48"/>
+      <c r="AA104" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="C127:D127"/>
-    <mergeCell ref="C122:D122"/>
-    <mergeCell ref="C123:D123"/>
-    <mergeCell ref="C124:D124"/>
-    <mergeCell ref="C125:D125"/>
-    <mergeCell ref="C126:D126"/>
+  <mergeCells count="10">
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="H7:K7"/>
     <mergeCell ref="A1:K1"/>
@@ -4064,6 +3622,7 @@
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
+    <mergeCell ref="C104:D104"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4089,16 +3648,16 @@
   <sheetData>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
       <c r="J8" s="11"/>
       <c r="K8" s="11" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
@@ -4106,46 +3665,46 @@
     </row>
     <row r="9" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F9" s="16" t="s">
+      <c r="G9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J9" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="G9" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J9" s="16" t="s">
-        <v>74</v>
-      </c>
       <c r="K9" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -4247,7 +3806,7 @@
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="4">
-        <f>'water tank'!D66/0.6</f>
+        <f>'water tank'!D56/0.6</f>
         <v>35.56666666666667</v>
       </c>
     </row>
@@ -4273,7 +3832,7 @@
         <v>4</v>
       </c>
       <c r="C87" s="3">
-        <f>'water tank'!D80</f>
+        <f>'water tank'!D68</f>
         <v>21.34</v>
       </c>
       <c r="D87" s="20">

</xml_diff>